<commit_message>
Document Claude handoff and record closing-bet no-trade review
</commit_message>
<xml_diff>
--- a/reference/종가베팅_거래기록_현재본.xlsx
+++ b/reference/종가베팅_거래기록_현재본.xlsx
@@ -2795,7 +2795,46 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>15:20</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>NO_TRADE</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="n">
+        <v>598280</v>
+      </c>
+      <c r="O6" t="n">
+        <v>598280</v>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>NO_TRADE</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>15:20:14 KRX 참고지수 코스피5556.31(-7.53%) 코스닥761.81(-7.53%); 시장 -3% 신규진입 차단 유지; PPI 발표 전 밤사이 위험; 추천 없음 0주 투자금0원 현금100%; 체결가 없음; 15:30 종가 아님; 사용자 실제거래·단타모의와 분리</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T4"/>
+  <autoFilter ref="A1:T6"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: preserve remaining analysis records and cross-PC handoff
</commit_message>
<xml_diff>
--- a/reference/종가베팅_거래기록_현재본.xlsx
+++ b/reference/종가베팅_거래기록_현재본.xlsx
@@ -2834,6 +2834,45 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>15:20</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>NO_TRADE</t>
+        </is>
+      </c>
+      <c r="H7">
+        <v>0</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="N7">
+        <v>598280</v>
+      </c>
+      <c r="O7">
+        <v>598280</v>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>NO_TRADE</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>2026-10-20 15:20:19 KST 확인; 지수 표시15:20:18 코스피5539.05(-3.97%) 코스닥781.84(-3.34%); 양시장상승목록재조회; 시장급락과 급등추격/기관프로그램촉매검증부족으로 NO_TRADE; 종목없음 0주 투자금0원 현금598280원100%; 개별체결가없음 15:30종가아님; 사용자토마토3400원18주실제매수는본AI모의와분리; 실제주문없음</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:T6"/>
 </worksheet>

</xml_diff>